<commit_message>
- Mejora de la lógica del modelo introduciendo explicitamente la existencia de slots "idle" donde no se llevan a cabo trabajos para tener en cuenta que los aviones deben ocupar posiciones mientras esperan posiciones. Incluyen restricciones adicionales para poder implementarlo así como para evitar superposiciones de slots. - Creación de un informe de solución donde se explicitan movimientos, duración de trabajos, retrasos por trabajo, por avión y por cliente. - Creación de case_3b en input_data.xlsx para poder comprobar funcionamiento de lógica de clientes.
</commit_message>
<xml_diff>
--- a/input_data.xlsx
+++ b/input_data.xlsx
@@ -1,25 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27126"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Mi unidad\academico\investigacion\proyectos\aircraft_positioning\codigo\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://upm365-my.sharepoint.com/personal/enrique_chbartol_alumnos_upm_es/Documents/UNIVERSIDAD/MASTER/TFM/CODE/aircraft-positioning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8BDC7DE-0FD8-4FE3-A3D5-C14737BF715F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="13_ncr:1_{A8BDC7DE-0FD8-4FE3-A3D5-C14737BF715F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B6ADBBD4-D687-40A7-9E42-8A674BA92D75}"/>
   <bookViews>
-    <workbookView xWindow="3840" yWindow="3840" windowWidth="23040" windowHeight="12120" activeTab="4" xr2:uid="{F5F6D73E-5AE2-4BF6-A18F-AC4E03A6BC3E}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{F5F6D73E-5AE2-4BF6-A18F-AC4E03A6BC3E}"/>
   </bookViews>
   <sheets>
     <sheet name="case_1_plane" sheetId="5" r:id="rId1"/>
     <sheet name="case_2_planes" sheetId="4" r:id="rId2"/>
     <sheet name="case_3_planes" sheetId="6" r:id="rId3"/>
-    <sheet name="case_4_planes" sheetId="7" r:id="rId4"/>
-    <sheet name="case_5_planes" sheetId="8" r:id="rId5"/>
-    <sheet name="case_2" sheetId="3" r:id="rId6"/>
-    <sheet name="use case1" sheetId="2" r:id="rId7"/>
+    <sheet name="case_3b_planes" sheetId="9" r:id="rId4"/>
+    <sheet name="case_4_planes" sheetId="7" r:id="rId5"/>
+    <sheet name="case_5_planes" sheetId="8" r:id="rId6"/>
+    <sheet name="case_2" sheetId="3" r:id="rId7"/>
+    <sheet name="use case1" sheetId="2" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="18">
   <si>
     <t xml:space="preserve">Avión </t>
   </si>
@@ -86,15 +87,30 @@
   <si>
     <t>duration</t>
   </si>
+  <si>
+    <t>client</t>
+  </si>
+  <si>
+    <t>Client 1</t>
+  </si>
+  <si>
+    <t>Client 2</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -143,9 +159,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -183,7 +199,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -289,7 +305,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -431,7 +447,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -978,6 +994,286 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{838F708A-CFA0-410F-9EA5-950802F67344}">
+  <dimension ref="A1:H10"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1" t="str">
+        <f>_xlfn.CONCAT(A2,"-",B2)</f>
+        <v>1-1</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <v>3</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3" s="1" t="str">
+        <f t="shared" ref="C3:C10" si="0">_xlfn.CONCAT(A3,"-",B3)</f>
+        <v>1-2</v>
+      </c>
+      <c r="D3">
+        <v>3</v>
+      </c>
+      <c r="E3">
+        <v>46</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>1</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>1-3</v>
+      </c>
+      <c r="D4">
+        <v>49</v>
+      </c>
+      <c r="E4">
+        <v>3</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="H4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>2</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>2-1</v>
+      </c>
+      <c r="D5">
+        <v>38</v>
+      </c>
+      <c r="E5">
+        <v>3</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="H5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>2</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>2-2</v>
+      </c>
+      <c r="D6">
+        <v>41</v>
+      </c>
+      <c r="E6">
+        <v>26</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>2</v>
+      </c>
+      <c r="B7">
+        <v>3</v>
+      </c>
+      <c r="C7" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>2-3</v>
+      </c>
+      <c r="D7">
+        <v>67</v>
+      </c>
+      <c r="E7">
+        <v>3</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="G7">
+        <v>1</v>
+      </c>
+      <c r="H7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>3</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>3-1</v>
+      </c>
+      <c r="D8">
+        <v>18</v>
+      </c>
+      <c r="E8">
+        <v>3</v>
+      </c>
+      <c r="F8">
+        <v>1</v>
+      </c>
+      <c r="G8">
+        <v>1</v>
+      </c>
+      <c r="H8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>3</v>
+      </c>
+      <c r="B9">
+        <v>2</v>
+      </c>
+      <c r="C9" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>3-2</v>
+      </c>
+      <c r="D9">
+        <v>21</v>
+      </c>
+      <c r="E9">
+        <v>37</v>
+      </c>
+      <c r="F9">
+        <v>0</v>
+      </c>
+      <c r="G9">
+        <v>1</v>
+      </c>
+      <c r="H9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>3</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>3-3</v>
+      </c>
+      <c r="D10">
+        <v>58</v>
+      </c>
+      <c r="E10">
+        <v>3</v>
+      </c>
+      <c r="F10">
+        <v>1</v>
+      </c>
+      <c r="G10">
+        <v>1</v>
+      </c>
+      <c r="H10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C81A5F7-0190-41C3-9890-78D02E0B8D1C}">
   <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1298,7 +1594,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A089C8E-0D83-467D-BA52-B2980240BDAD}">
   <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1691,7 +1987,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3857537-A0B6-4891-B116-ACB4B38341D3}">
   <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2160,7 +2456,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26AEF585-7FE3-4F9A-B091-89E2D051FC68}">
   <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
- Actualización de la función check_solution que ahora incluye la verificación de las nuevas restricciones. - Cambio en el nombre de la hoja con 6 aviones en el excel de input de datos
</commit_message>
<xml_diff>
--- a/input_data.xlsx
+++ b/input_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://upm365-my.sharepoint.com/personal/enrique_chbartol_alumnos_upm_es/Documents/UNIVERSIDAD/MASTER/TFM/CODE/aircraft-positioning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="13_ncr:1_{A8BDC7DE-0FD8-4FE3-A3D5-C14737BF715F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B6ADBBD4-D687-40A7-9E42-8A674BA92D75}"/>
+  <xr:revisionPtr revIDLastSave="43" documentId="13_ncr:1_{A8BDC7DE-0FD8-4FE3-A3D5-C14737BF715F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{79BC1C73-2345-4C5B-8DC0-73FF0EE60E24}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{F5F6D73E-5AE2-4BF6-A18F-AC4E03A6BC3E}"/>
+    <workbookView xWindow="34935" yWindow="6120" windowWidth="17280" windowHeight="8880" firstSheet="4" activeTab="7" xr2:uid="{F5F6D73E-5AE2-4BF6-A18F-AC4E03A6BC3E}"/>
   </bookViews>
   <sheets>
     <sheet name="case_1_plane" sheetId="5" r:id="rId1"/>
@@ -19,8 +19,9 @@
     <sheet name="case_3b_planes" sheetId="9" r:id="rId4"/>
     <sheet name="case_4_planes" sheetId="7" r:id="rId5"/>
     <sheet name="case_5_planes" sheetId="8" r:id="rId6"/>
-    <sheet name="case_2" sheetId="3" r:id="rId7"/>
-    <sheet name="use case1" sheetId="2" r:id="rId8"/>
+    <sheet name="case_6_planes" sheetId="3" r:id="rId7"/>
+    <sheet name="Planes" sheetId="10" r:id="rId8"/>
+    <sheet name="use case1" sheetId="2" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="20">
   <si>
     <t xml:space="preserve">Avión </t>
   </si>
@@ -95,6 +96,12 @@
   </si>
   <si>
     <t>Client 2</t>
+  </si>
+  <si>
+    <t>early_start</t>
+  </si>
+  <si>
+    <t>late_finish_deadline</t>
   </si>
 </sst>
 </file>
@@ -2453,10 +2460,98 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7F3BC76-AA2A-435F-948E-0EB92929D05D}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>38</v>
+      </c>
+      <c r="C3">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>10</v>
+      </c>
+      <c r="C4">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>45</v>
+      </c>
+      <c r="C5">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>50</v>
+      </c>
+      <c r="C6">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>56</v>
+      </c>
+      <c r="C7">
+        <v>84</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26AEF585-7FE3-4F9A-B091-89E2D051FC68}">
   <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>